<commit_message>
fix: correct JSON keys and repopulate all Pitches column entries
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEO/outreach-targets.xlsx
+++ b/SEO/outreach-targets.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1178" uniqueCount="599">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1301" uniqueCount="606">
   <si>
     <t>Name</t>
   </si>
@@ -792,6 +792,13 @@
     <t>Canon/Nikon/Sony audience. HEIC format guides are huge here.</t>
   </si>
   <si>
+    <t xml:space="preserve">Subject: Local-first HEIC batch converter — reader tool worth knowing about
+Hi dpreview editorial team,
+dpreview readers regularly ask how to batch-convert HEIC files from iPhones without pushing personal photos to a cloud service. ConvertYard does this entirely in the browser via WebAssembly — no server, no account, supports JPG, WebP, and AVIF output. It handles 1000+ files in a single batch. Worth a mention in your software/workflow coverage if you're covering HEIC tools this cycle.
+— Garrick
+convertyard.com</t>
+  </si>
+  <si>
     <t>iMore</t>
   </si>
   <si>
@@ -802,6 +809,14 @@
   </si>
   <si>
     <t>Apple/iPhone audience. "How to convert HEIC to JPG on iPhone/Mac" articles are very popular.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subject: Free batch HEIC converter — browser-only, no iCloud required
+Hi [MacRumors/AppleInsider] team,
+iPhone users shooting HEIC by default still hit a wall when sharing photos with Windows users or uploading to sites that reject the format. ConvertYard converts batches of HEIC files to JPG or WebP in the browser via WebAssembly — no iCloud, no server upload, no account, works on any OS. Drop 500 photos, download a ZIP of JPGs in seconds. Worth a tip post if you're covering HEIC workarounds this month.
+(Note: iMore shut down July 16, 2026 — send to tips@macrumors.com or news@appleinsider.com instead.)
+— Garrick
+convertyard.com</t>
   </si>
   <si>
     <t>9to5Mac</t>
@@ -946,6 +961,13 @@
     <t>Dev tools roundups. Very high DA. Pitch the JSON formatter / diff checker.</t>
   </si>
   <si>
+    <t xml:space="preserve">Subject: Zero server requests: running 93 file converters entirely in WASM
+Hi CSS-Tricks team,
+Your recent "What's !important #15" roundup caught my attention — you cover the browser platform deeply, and I think ConvertYard fits squarely in that territory. I built a batch file converter (93 tools: images, PDF, video, audio) where every conversion runs client-side via ffmpeg.wasm, libvips-wasm, mupdf-wasm, and transformers.js — open DevTools during a conversion and you'll see zero outgoing network requests. I'd love to write a deep-dive guest article on architecting zero-server file processing with WebAssembly for the CSS-Tricks audience.
+— Garrick
+convertyard.com</t>
+  </si>
+  <si>
     <t>DZone</t>
   </si>
   <si>
@@ -1293,6 +1315,13 @@
     <t>Accessibility audience. alt-text-generator as a free tool for making images accessible.</t>
   </si>
   <si>
+    <t xml:space="preserve">Subject: Free local OCR for inaccessible PDFs and scanned documents
+Hi WebAIM team,
+Your recent post on accessibility extensions made a point that stuck with me: remediating old inaccessible PDFs while publishing new inaccessible ones is "bailing water with the faucet still running." One practical piece of that remediation is extracting text from scanned documents and image-based PDFs. I built a free browser-based OCR tool (screenshot-to-text, image-to-Excel) that runs entirely on-device via transformers.js — no upload, no account — so organizations can extract text from legacy scanned files without sending sensitive documents to a cloud service. Worth a mention in your resources or tools coverage if it fits.
+— Garrick
+convertyard.com</t>
+  </si>
+  <si>
     <t>A11y Project</t>
   </si>
   <si>
@@ -1394,6 +1423,13 @@
     <t>Creator economy coverage. Free tools for video creators.</t>
   </si>
   <si>
+    <t xml:space="preserve">Subject: A free, private browser tool for music creators handling their own files
+Hi Dan,
+Your piece on AI and human creativity cuts close to what independent artists deal with daily: doing more with less, while keeping control of their work. ConvertYard is a set of browser-based audio and video tools — MP4 to MP3, audio trimmer, video compressor — that run entirely via ffmpeg.wasm. No upload, no watermark, no subscription. For artists handling client or unreleased material, that privacy is non-negotiable. If it fits a future piece on creator tools, happy to talk.
+— Garrick
+convertyard.com</t>
+  </si>
+  <si>
     <t>Ben's Bites</t>
   </si>
   <si>
@@ -1471,6 +1507,12 @@
   </si>
   <si>
     <t>Schedule a second PH launch focused on AI tools cluster.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subject: ConvertYard — browser-local AI inference for file conversion, no API key needed
+ConvertYard runs AI-powered tools (OCR, alt-text generation, background removal, handwriting recognition, image-to-Excel) entirely in the browser via transformers.js and WebAssembly. No file ever leaves your device — open DevTools during a conversion and the Network tab stays empty. 93 tools total, batch up to 1,000 files, no account required.
+Launching as an AI product because the local inference story is what makes it genuinely different from every other "AI-powered" converter that quietly ships your files to a cloud API.
+convertyard.com</t>
   </si>
   <si>
     <t>Every.to</t>
@@ -1572,6 +1614,9 @@
   </si>
   <si>
     <t>Daily design links. Share the color-picker or gradient-generator.</t>
+  </si>
+  <si>
+    <t>ConvertYard is a local-first batch file converter — 93 tools, everything in WebAssembly, zero outgoing network requests during conversion, up to 1,000 files at a time: convertyard.com</t>
   </si>
   <si>
     <t>Hacker News — Show HN</t>
@@ -2384,7 +2429,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J35"/>
-  <sheetFormatPr customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
@@ -3422,8 +3467,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K63"/>
-  <sheetFormatPr customHeight="1"/>
+  <dimension ref="A1:M63"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
@@ -3437,7 +3482,7 @@
     <col min="10" max="10" width="70.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3471,8 +3516,14 @@
       <c r="K1" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>163</v>
       </c>
@@ -3500,8 +3551,14 @@
       <c r="K2" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" t="s">
+        <v>169</v>
+      </c>
+      <c r="M2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>170</v>
       </c>
@@ -3529,8 +3586,14 @@
       <c r="K3" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" t="s">
+        <v>174</v>
+      </c>
+      <c r="M3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>175</v>
       </c>
@@ -3558,8 +3621,14 @@
       <c r="K4" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" t="s">
+        <v>179</v>
+      </c>
+      <c r="M4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>180</v>
       </c>
@@ -3587,8 +3656,14 @@
       <c r="K5" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" t="s">
+        <v>184</v>
+      </c>
+      <c r="M5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>185</v>
       </c>
@@ -3616,8 +3691,14 @@
       <c r="K6" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6" t="s">
+        <v>189</v>
+      </c>
+      <c r="M6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>190</v>
       </c>
@@ -3645,8 +3726,14 @@
       <c r="K7" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7" t="s">
+        <v>194</v>
+      </c>
+      <c r="M7" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>195</v>
       </c>
@@ -3674,8 +3761,14 @@
       <c r="K8" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" t="s">
+        <v>199</v>
+      </c>
+      <c r="M8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>200</v>
       </c>
@@ -3703,8 +3796,14 @@
       <c r="K9" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9" t="s">
+        <v>204</v>
+      </c>
+      <c r="M9" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>205</v>
       </c>
@@ -3732,8 +3831,14 @@
       <c r="K10" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" t="s">
+        <v>209</v>
+      </c>
+      <c r="M10" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>210</v>
       </c>
@@ -3761,8 +3866,14 @@
       <c r="K11" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L11" t="s">
+        <v>214</v>
+      </c>
+      <c r="M11" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>215</v>
       </c>
@@ -3790,8 +3901,14 @@
       <c r="K12" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L12" t="s">
+        <v>219</v>
+      </c>
+      <c r="M12" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>220</v>
       </c>
@@ -3819,8 +3936,14 @@
       <c r="K13" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13" t="s">
+        <v>224</v>
+      </c>
+      <c r="M13" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>225</v>
       </c>
@@ -3848,8 +3971,14 @@
       <c r="K14" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L14" t="s">
+        <v>230</v>
+      </c>
+      <c r="M14" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>231</v>
       </c>
@@ -3877,8 +4006,14 @@
       <c r="K15" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L15" t="s">
+        <v>235</v>
+      </c>
+      <c r="M15" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>236</v>
       </c>
@@ -3903,13 +4038,19 @@
       <c r="J16" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L16" t="s">
+        <v>240</v>
+      </c>
+      <c r="M16" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B17" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C17" t="s">
         <v>227</v>
@@ -3921,21 +4062,27 @@
         <v>14</v>
       </c>
       <c r="F17" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G17" t="s">
         <v>132</v>
       </c>
       <c r="J17" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+        <v>244</v>
+      </c>
+      <c r="L17" t="s">
+        <v>245</v>
+      </c>
+      <c r="M17" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B18" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C18" t="s">
         <v>227</v>
@@ -3947,24 +4094,30 @@
         <v>14</v>
       </c>
       <c r="F18" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G18" t="s">
         <v>132</v>
       </c>
       <c r="J18" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="K18" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+      <c r="L18" t="s">
+        <v>250</v>
+      </c>
+      <c r="M18" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B19" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C19" t="s">
         <v>227</v>
@@ -3976,24 +4129,30 @@
         <v>14</v>
       </c>
       <c r="F19" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="G19" t="s">
         <v>132</v>
       </c>
       <c r="J19" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="K19" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+        <v>255</v>
+      </c>
+      <c r="L19" t="s">
+        <v>255</v>
+      </c>
+      <c r="M19" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B20" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C20" t="s">
         <v>227</v>
@@ -4011,18 +4170,24 @@
         <v>132</v>
       </c>
       <c r="J20" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="K20" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+        <v>259</v>
+      </c>
+      <c r="L20" t="s">
+        <v>259</v>
+      </c>
+      <c r="M20" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B21" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C21" t="s">
         <v>227</v>
@@ -4034,24 +4199,30 @@
         <v>55</v>
       </c>
       <c r="F21" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="G21" t="s">
         <v>132</v>
       </c>
       <c r="J21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="K21" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+        <v>264</v>
+      </c>
+      <c r="L21" t="s">
+        <v>264</v>
+      </c>
+      <c r="M21" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B22" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C22" t="s">
         <v>227</v>
@@ -4063,24 +4234,30 @@
         <v>55</v>
       </c>
       <c r="F22" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G22" t="s">
         <v>132</v>
       </c>
       <c r="J22" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="K22" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+        <v>269</v>
+      </c>
+      <c r="L22" t="s">
+        <v>269</v>
+      </c>
+      <c r="M22" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B23" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C23" t="s">
         <v>227</v>
@@ -4092,24 +4269,30 @@
         <v>55</v>
       </c>
       <c r="F23" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="G23" t="s">
         <v>132</v>
       </c>
       <c r="J23" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="K23" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+        <v>274</v>
+      </c>
+      <c r="L23" t="s">
+        <v>274</v>
+      </c>
+      <c r="M23" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B24" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C24" t="s">
         <v>227</v>
@@ -4121,24 +4304,30 @@
         <v>55</v>
       </c>
       <c r="F24" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="G24" t="s">
         <v>132</v>
       </c>
       <c r="J24" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="K24" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+        <v>279</v>
+      </c>
+      <c r="L24" t="s">
+        <v>279</v>
+      </c>
+      <c r="M24" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B25" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C25" t="s">
         <v>127</v>
@@ -4150,21 +4339,27 @@
         <v>14</v>
       </c>
       <c r="F25" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="G25" t="s">
         <v>132</v>
       </c>
       <c r="J25" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+        <v>283</v>
+      </c>
+      <c r="L25" t="s">
+        <v>284</v>
+      </c>
+      <c r="M25" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B26" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C26" t="s">
         <v>127</v>
@@ -4176,24 +4371,30 @@
         <v>14</v>
       </c>
       <c r="F26" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="G26" t="s">
         <v>132</v>
       </c>
       <c r="J26" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="K26" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+        <v>289</v>
+      </c>
+      <c r="L26" t="s">
+        <v>289</v>
+      </c>
+      <c r="M26" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B27" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C27" t="s">
         <v>127</v>
@@ -4205,24 +4406,30 @@
         <v>55</v>
       </c>
       <c r="F27" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="G27" t="s">
         <v>132</v>
       </c>
       <c r="J27" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="K27" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+        <v>291</v>
+      </c>
+      <c r="L27" t="s">
+        <v>291</v>
+      </c>
+      <c r="M27" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B28" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C28" t="s">
         <v>127</v>
@@ -4234,24 +4441,30 @@
         <v>55</v>
       </c>
       <c r="F28" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="G28" t="s">
         <v>132</v>
       </c>
       <c r="J28" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="K28" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+        <v>296</v>
+      </c>
+      <c r="L28" t="s">
+        <v>296</v>
+      </c>
+      <c r="M28" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B29" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C29" t="s">
         <v>127</v>
@@ -4263,24 +4476,30 @@
         <v>14</v>
       </c>
       <c r="F29" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="G29" t="s">
         <v>153</v>
       </c>
       <c r="J29" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="K29" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+        <v>301</v>
+      </c>
+      <c r="L29" t="s">
+        <v>301</v>
+      </c>
+      <c r="M29" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B30" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C30" t="s">
         <v>127</v>
@@ -4292,24 +4511,30 @@
         <v>55</v>
       </c>
       <c r="F30" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="G30" t="s">
         <v>153</v>
       </c>
       <c r="J30" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="K30" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+      <c r="L30" t="s">
+        <v>306</v>
+      </c>
+      <c r="M30" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B31" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C31" t="s">
         <v>127</v>
@@ -4321,280 +4546,340 @@
         <v>55</v>
       </c>
       <c r="F31" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="G31" t="s">
         <v>132</v>
       </c>
       <c r="J31" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="K31" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+        <v>311</v>
+      </c>
+      <c r="L31" t="s">
+        <v>311</v>
+      </c>
+      <c r="M31" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B32" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="C32" t="s">
         <v>127</v>
       </c>
       <c r="D32" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E32" t="s">
         <v>14</v>
       </c>
       <c r="F32" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="G32" t="s">
         <v>132</v>
       </c>
       <c r="J32" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="K32" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+        <v>317</v>
+      </c>
+      <c r="L32" t="s">
+        <v>317</v>
+      </c>
+      <c r="M32" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B33" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C33" t="s">
         <v>127</v>
       </c>
       <c r="D33" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E33" t="s">
         <v>55</v>
       </c>
       <c r="F33" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="G33" t="s">
         <v>132</v>
       </c>
       <c r="J33" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="K33" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+        <v>322</v>
+      </c>
+      <c r="L33" t="s">
+        <v>322</v>
+      </c>
+      <c r="M33" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B34" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C34" t="s">
         <v>127</v>
       </c>
       <c r="D34" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E34" t="s">
         <v>14</v>
       </c>
       <c r="F34" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="G34" t="s">
         <v>132</v>
       </c>
       <c r="J34" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="K34" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+        <v>327</v>
+      </c>
+      <c r="L34" t="s">
+        <v>327</v>
+      </c>
+      <c r="M34" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B35" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C35" t="s">
         <v>127</v>
       </c>
       <c r="D35" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E35" t="s">
         <v>14</v>
       </c>
       <c r="F35" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="G35" t="s">
         <v>132</v>
       </c>
       <c r="J35" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="K35" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+        <v>332</v>
+      </c>
+      <c r="L35" t="s">
+        <v>332</v>
+      </c>
+      <c r="M35" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B36" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="C36" t="s">
         <v>127</v>
       </c>
       <c r="D36" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="E36" t="s">
         <v>55</v>
       </c>
       <c r="F36" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="G36" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="J36" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="K36" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+      <c r="L36" t="s">
+        <v>339</v>
+      </c>
+      <c r="M36" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B37" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C37" t="s">
         <v>127</v>
       </c>
       <c r="D37" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="E37" t="s">
         <v>55</v>
       </c>
       <c r="F37" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="G37" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="J37" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="K37" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+        <v>344</v>
+      </c>
+      <c r="L37" t="s">
+        <v>344</v>
+      </c>
+      <c r="M37" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B38" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C38" t="s">
         <v>127</v>
       </c>
       <c r="D38" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="E38" t="s">
         <v>55</v>
       </c>
       <c r="F38" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="G38" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="J38" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="K38" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+      <c r="L38" t="s">
+        <v>349</v>
+      </c>
+      <c r="M38" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B39" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C39" t="s">
         <v>127</v>
       </c>
       <c r="D39" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E39" t="s">
         <v>55</v>
       </c>
       <c r="F39" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="G39" t="s">
         <v>132</v>
       </c>
       <c r="J39" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="K39" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+        <v>353</v>
+      </c>
+      <c r="L39" t="s">
+        <v>353</v>
+      </c>
+      <c r="M39" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B40" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C40" t="s">
         <v>127</v>
       </c>
       <c r="D40" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E40" t="s">
         <v>14</v>
       </c>
       <c r="F40" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="G40" t="s">
         <v>153</v>
       </c>
       <c r="J40" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="K40" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+        <v>358</v>
+      </c>
+      <c r="L40" t="s">
+        <v>358</v>
+      </c>
+      <c r="M40" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>215</v>
       </c>
@@ -4602,7 +4887,7 @@
         <v>216</v>
       </c>
       <c r="C41" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D41" t="s">
         <v>166</v>
@@ -4617,13 +4902,19 @@
         <v>132</v>
       </c>
       <c r="J41" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="K41" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+        <v>361</v>
+      </c>
+      <c r="L41" t="s">
+        <v>361</v>
+      </c>
+      <c r="M41" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>180</v>
       </c>
@@ -4631,7 +4922,7 @@
         <v>181</v>
       </c>
       <c r="C42" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D42" t="s">
         <v>166</v>
@@ -4640,27 +4931,33 @@
         <v>14</v>
       </c>
       <c r="F42" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="G42" t="s">
         <v>132</v>
       </c>
       <c r="J42" t="s">
+        <v>362</v>
+      </c>
+      <c r="K42" t="s">
+        <v>363</v>
+      </c>
+      <c r="L42" t="s">
+        <v>363</v>
+      </c>
+      <c r="M42" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>364</v>
+      </c>
+      <c r="B43" t="s">
+        <v>365</v>
+      </c>
+      <c r="C43" t="s">
         <v>359</v>
-      </c>
-      <c r="K42" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>361</v>
-      </c>
-      <c r="B43" t="s">
-        <v>362</v>
-      </c>
-      <c r="C43" t="s">
-        <v>356</v>
       </c>
       <c r="D43" t="s">
         <v>166</v>
@@ -4669,27 +4966,33 @@
         <v>55</v>
       </c>
       <c r="F43" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="G43" t="s">
         <v>132</v>
       </c>
       <c r="J43" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="K43" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+        <v>368</v>
+      </c>
+      <c r="L43" t="s">
+        <v>368</v>
+      </c>
+      <c r="M43" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="B44" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C44" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D44" t="s">
         <v>158</v>
@@ -4698,27 +5001,33 @@
         <v>55</v>
       </c>
       <c r="F44" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="G44" t="s">
         <v>153</v>
       </c>
       <c r="J44" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="K44" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+        <v>373</v>
+      </c>
+      <c r="L44" t="s">
+        <v>373</v>
+      </c>
+      <c r="M44" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B45" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C45" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D45" t="s">
         <v>158</v>
@@ -4727,27 +5036,33 @@
         <v>55</v>
       </c>
       <c r="F45" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="G45" t="s">
         <v>153</v>
       </c>
       <c r="J45" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="K45" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+      <c r="L45" t="s">
+        <v>378</v>
+      </c>
+      <c r="M45" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B46" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="C46" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D46" t="s">
         <v>166</v>
@@ -4762,18 +5077,21 @@
         <v>132</v>
       </c>
       <c r="J46" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+      <c r="M46" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="B47" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="C47" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D47" t="s">
         <v>166</v>
@@ -4782,27 +5100,33 @@
         <v>97</v>
       </c>
       <c r="F47" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="G47" t="s">
         <v>132</v>
       </c>
       <c r="J47" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="K47" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+      <c r="L47" t="s">
+        <v>387</v>
+      </c>
+      <c r="M47" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="B48" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="C48" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D48" t="s">
         <v>166</v>
@@ -4817,21 +5141,27 @@
         <v>132</v>
       </c>
       <c r="J48" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="K48" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+        <v>392</v>
+      </c>
+      <c r="L48" t="s">
+        <v>392</v>
+      </c>
+      <c r="M48" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="B49" t="s">
+        <v>394</v>
+      </c>
+      <c r="C49" t="s">
         <v>390</v>
-      </c>
-      <c r="C49" t="s">
-        <v>386</v>
       </c>
       <c r="D49" t="s">
         <v>166</v>
@@ -4840,27 +5170,33 @@
         <v>14</v>
       </c>
       <c r="F49" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="G49" t="s">
         <v>132</v>
       </c>
       <c r="J49" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="K49" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+        <v>397</v>
+      </c>
+      <c r="L49" t="s">
+        <v>397</v>
+      </c>
+      <c r="M49" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="B50" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="C50" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D50" t="s">
         <v>166</v>
@@ -4869,27 +5205,33 @@
         <v>55</v>
       </c>
       <c r="F50" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="G50" t="s">
         <v>132</v>
       </c>
       <c r="J50" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="K50" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+        <v>401</v>
+      </c>
+      <c r="L50" t="s">
+        <v>401</v>
+      </c>
+      <c r="M50" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="B51" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="C51" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D51" t="s">
         <v>166</v>
@@ -4904,128 +5246,155 @@
         <v>132</v>
       </c>
       <c r="J51" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="K51" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+      <c r="L51" t="s">
+        <v>405</v>
+      </c>
+      <c r="M51" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B52" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C52" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D52" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E52" t="s">
         <v>97</v>
       </c>
       <c r="F52" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="G52" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="J52" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+      <c r="M52" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="B53" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="C53" t="s">
         <v>42</v>
       </c>
       <c r="D53" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E53" t="s">
         <v>14</v>
       </c>
       <c r="F53" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="G53" t="s">
         <v>132</v>
       </c>
       <c r="J53" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="K53" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+        <v>415</v>
+      </c>
+      <c r="L53" t="s">
+        <v>415</v>
+      </c>
+      <c r="M53" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="B54" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="C54" t="s">
         <v>42</v>
       </c>
       <c r="D54" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E54" t="s">
         <v>14</v>
       </c>
       <c r="F54" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="G54" t="s">
         <v>132</v>
       </c>
       <c r="J54" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="K54" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+      <c r="L54" t="s">
+        <v>420</v>
+      </c>
+      <c r="M54" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="B55" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="C55" t="s">
         <v>42</v>
       </c>
       <c r="D55" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E55" t="s">
         <v>14</v>
       </c>
       <c r="F55" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="G55" t="s">
         <v>132</v>
       </c>
       <c r="J55" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="K55" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+        <v>424</v>
+      </c>
+      <c r="L55" t="s">
+        <v>424</v>
+      </c>
+      <c r="M55" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="B56" t="s">
         <v>41</v>
@@ -5034,30 +5403,36 @@
         <v>42</v>
       </c>
       <c r="D56" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E56" t="s">
         <v>55</v>
       </c>
       <c r="F56" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="G56" t="s">
         <v>132</v>
       </c>
       <c r="J56" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="K56" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+        <v>428</v>
+      </c>
+      <c r="L56" t="s">
+        <v>428</v>
+      </c>
+      <c r="M56" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="B57" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="C57" t="s">
         <v>42</v>
@@ -5075,178 +5450,217 @@
         <v>132</v>
       </c>
       <c r="J57" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+      <c r="M57" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="B58" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
       <c r="C58" t="s">
         <v>42</v>
       </c>
       <c r="D58" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E58" t="s">
         <v>55</v>
       </c>
       <c r="F58" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="G58" t="s">
         <v>132</v>
       </c>
       <c r="J58" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="K58" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+        <v>437</v>
+      </c>
+      <c r="L58" t="s">
+        <v>437</v>
+      </c>
+      <c r="M58" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="B59" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="C59" t="s">
         <v>42</v>
       </c>
       <c r="D59" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E59" t="s">
         <v>97</v>
       </c>
       <c r="F59" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="G59" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="J59" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="K59" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+        <v>442</v>
+      </c>
+      <c r="L59" t="s">
+        <v>442</v>
+      </c>
+      <c r="M59" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="B60" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="C60" t="s">
         <v>12</v>
       </c>
       <c r="D60" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E60" t="s">
         <v>14</v>
       </c>
       <c r="F60" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="G60" t="s">
         <v>153</v>
       </c>
       <c r="J60" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="K60" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+        <v>447</v>
+      </c>
+      <c r="L60" t="s">
+        <v>447</v>
+      </c>
+      <c r="M60" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="B61" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="C61" t="s">
         <v>12</v>
       </c>
       <c r="D61" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E61" t="s">
         <v>55</v>
       </c>
       <c r="F61" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="G61" t="s">
         <v>132</v>
       </c>
       <c r="J61" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="K61" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+        <v>452</v>
+      </c>
+      <c r="L61" t="s">
+        <v>452</v>
+      </c>
+      <c r="M61" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="B62" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="C62" t="s">
         <v>12</v>
       </c>
       <c r="D62" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E62" t="s">
         <v>55</v>
       </c>
       <c r="F62" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="G62" t="s">
         <v>132</v>
       </c>
       <c r="J62" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="K62" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+        <v>457</v>
+      </c>
+      <c r="L62" t="s">
+        <v>457</v>
+      </c>
+      <c r="M62" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="B63" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="C63" t="s">
         <v>127</v>
       </c>
       <c r="D63" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E63" t="s">
         <v>55</v>
       </c>
       <c r="F63" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="G63" t="s">
         <v>153</v>
       </c>
       <c r="J63" t="s">
-        <v>454</v>
+        <v>460</v>
+      </c>
+      <c r="L63" t="s">
+        <v>461</v>
+      </c>
+      <c r="M63" t="s">
+        <v>461</v>
       </c>
     </row>
   </sheetData>
@@ -5256,7 +5670,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J30"/>
-  <sheetFormatPr customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
@@ -5304,10 +5718,10 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="B2" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -5319,13 +5733,13 @@
         <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="G2" t="s">
         <v>153</v>
       </c>
       <c r="J2" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -5351,15 +5765,15 @@
         <v>153</v>
       </c>
       <c r="J3" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="B4" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="C4" t="s">
         <v>127</v>
@@ -5371,21 +5785,21 @@
         <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G4" t="s">
         <v>153</v>
       </c>
       <c r="J4" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="B5" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
@@ -5397,21 +5811,21 @@
         <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G5" t="s">
         <v>153</v>
       </c>
       <c r="J5" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="B6" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
       <c r="C6" t="s">
         <v>12</v>
@@ -5423,21 +5837,21 @@
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G6" t="s">
         <v>153</v>
       </c>
       <c r="J6" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="B7" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="C7" t="s">
         <v>165</v>
@@ -5449,21 +5863,21 @@
         <v>14</v>
       </c>
       <c r="F7" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G7" t="s">
         <v>153</v>
       </c>
       <c r="J7" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="B8" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="C8" t="s">
         <v>227</v>
@@ -5475,24 +5889,24 @@
         <v>55</v>
       </c>
       <c r="F8" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G8" t="s">
         <v>153</v>
       </c>
       <c r="J8" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="B9" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="C9" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D9" t="s">
         <v>158</v>
@@ -5501,21 +5915,21 @@
         <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G9" t="s">
         <v>153</v>
       </c>
       <c r="J9" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="B10" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -5527,21 +5941,21 @@
         <v>55</v>
       </c>
       <c r="F10" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G10" t="s">
         <v>153</v>
       </c>
       <c r="J10" t="s">
-        <v>481</v>
+        <v>488</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="B11" t="s">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="C11" t="s">
         <v>42</v>
@@ -5553,21 +5967,21 @@
         <v>97</v>
       </c>
       <c r="F11" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G11" t="s">
         <v>153</v>
       </c>
       <c r="J11" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
       <c r="B12" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="C12" t="s">
         <v>165</v>
@@ -5579,24 +5993,24 @@
         <v>55</v>
       </c>
       <c r="F12" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
       <c r="G12" t="s">
         <v>132</v>
       </c>
       <c r="J12" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B13" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C13" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D13" t="s">
         <v>158</v>
@@ -5605,24 +6019,24 @@
         <v>55</v>
       </c>
       <c r="F13" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="G13" t="s">
         <v>153</v>
       </c>
       <c r="J13" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="B14" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
       <c r="C14" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="D14" t="s">
         <v>158</v>
@@ -5631,24 +6045,24 @@
         <v>55</v>
       </c>
       <c r="F14" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G14" t="s">
         <v>153</v>
       </c>
       <c r="J14" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>493</v>
+        <v>500</v>
       </c>
       <c r="B15" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
       <c r="C15" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D15" t="s">
         <v>158</v>
@@ -5657,21 +6071,21 @@
         <v>97</v>
       </c>
       <c r="F15" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G15" t="s">
         <v>153</v>
       </c>
       <c r="J15" t="s">
-        <v>495</v>
+        <v>502</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
       <c r="B16" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
       <c r="C16" t="s">
         <v>42</v>
@@ -5683,21 +6097,21 @@
         <v>97</v>
       </c>
       <c r="F16" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G16" t="s">
         <v>153</v>
       </c>
       <c r="J16" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B17" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C17" t="s">
         <v>127</v>
@@ -5709,21 +6123,21 @@
         <v>14</v>
       </c>
       <c r="F17" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
       <c r="G17" t="s">
         <v>153</v>
       </c>
       <c r="J17" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B18" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C18" t="s">
         <v>127</v>
@@ -5735,21 +6149,21 @@
         <v>55</v>
       </c>
       <c r="F18" t="s">
-        <v>501</v>
+        <v>508</v>
       </c>
       <c r="G18" t="s">
         <v>153</v>
       </c>
       <c r="J18" t="s">
-        <v>502</v>
+        <v>509</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>503</v>
+        <v>510</v>
       </c>
       <c r="B19" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="C19" t="s">
         <v>127</v>
@@ -5761,21 +6175,21 @@
         <v>14</v>
       </c>
       <c r="F19" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G19" t="s">
         <v>153</v>
       </c>
       <c r="J19" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B20" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C20" t="s">
         <v>127</v>
@@ -5787,13 +6201,13 @@
         <v>55</v>
       </c>
       <c r="F20" t="s">
-        <v>506</v>
+        <v>513</v>
       </c>
       <c r="G20" t="s">
         <v>132</v>
       </c>
       <c r="J20" t="s">
-        <v>507</v>
+        <v>514</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -5813,21 +6227,21 @@
         <v>14</v>
       </c>
       <c r="F21" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="G21" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="J21" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="B22" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -5839,21 +6253,21 @@
         <v>97</v>
       </c>
       <c r="F22" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="G22" t="s">
         <v>132</v>
       </c>
       <c r="J22" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B23" t="s">
-        <v>515</v>
+        <v>522</v>
       </c>
       <c r="C23" t="s">
         <v>12</v>
@@ -5865,21 +6279,21 @@
         <v>97</v>
       </c>
       <c r="F23" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="G23" t="s">
         <v>16</v>
       </c>
       <c r="J23" t="s">
-        <v>517</v>
+        <v>524</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="B24" t="s">
-        <v>519</v>
+        <v>526</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
@@ -5891,21 +6305,21 @@
         <v>55</v>
       </c>
       <c r="F24" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
       <c r="G24" t="s">
-        <v>521</v>
+        <v>528</v>
       </c>
       <c r="J24" t="s">
-        <v>522</v>
+        <v>529</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="B25" t="s">
-        <v>519</v>
+        <v>526</v>
       </c>
       <c r="C25" t="s">
         <v>127</v>
@@ -5917,21 +6331,21 @@
         <v>55</v>
       </c>
       <c r="F25" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
       <c r="G25" t="s">
         <v>153</v>
       </c>
       <c r="J25" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="B26" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -5943,21 +6357,21 @@
         <v>14</v>
       </c>
       <c r="F26" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
       <c r="G26" t="s">
         <v>132</v>
       </c>
       <c r="J26" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
       <c r="B27" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
       <c r="C27" t="s">
         <v>12</v>
@@ -5969,21 +6383,21 @@
         <v>14</v>
       </c>
       <c r="F27" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
       <c r="G27" t="s">
         <v>132</v>
       </c>
       <c r="J27" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="B28" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
       <c r="C28" t="s">
         <v>12</v>
@@ -5995,24 +6409,24 @@
         <v>55</v>
       </c>
       <c r="F28" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="G28" t="s">
         <v>132</v>
       </c>
       <c r="J28" t="s">
-        <v>536</v>
+        <v>543</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="B29" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C29" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D29" t="s">
         <v>158</v>
@@ -6021,21 +6435,21 @@
         <v>55</v>
       </c>
       <c r="F29" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
       <c r="G29" t="s">
         <v>153</v>
       </c>
       <c r="J29" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>539</v>
+        <v>546</v>
       </c>
       <c r="B30" t="s">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="C30" t="s">
         <v>127</v>
@@ -6047,13 +6461,13 @@
         <v>97</v>
       </c>
       <c r="F30" t="s">
-        <v>541</v>
+        <v>548</v>
       </c>
       <c r="G30" t="s">
         <v>132</v>
       </c>
       <c r="J30" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
     </row>
   </sheetData>
@@ -6063,7 +6477,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C24"/>
-  <sheetFormatPr customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -6072,216 +6486,216 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>543</v>
+        <v>550</v>
       </c>
       <c r="B1" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="C1" t="s">
-        <v>545</v>
+        <v>552</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="B3" t="s">
         <v>60</v>
       </c>
       <c r="C3" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>550</v>
+        <v>557</v>
       </c>
       <c r="B4" t="s">
-        <v>551</v>
+        <v>558</v>
       </c>
       <c r="C4" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="B5" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
       <c r="C5" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>556</v>
+        <v>563</v>
       </c>
       <c r="B7" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
       <c r="C7" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>559</v>
+        <v>566</v>
       </c>
       <c r="B9" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
       <c r="C9" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>562</v>
+        <v>569</v>
       </c>
       <c r="B11" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
       <c r="C11" t="s">
-        <v>564</v>
+        <v>571</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
       <c r="B12" t="s">
-        <v>566</v>
+        <v>573</v>
       </c>
       <c r="C12" t="s">
-        <v>567</v>
+        <v>574</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>568</v>
+        <v>575</v>
       </c>
       <c r="B13" t="s">
-        <v>569</v>
+        <v>576</v>
       </c>
       <c r="C13" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="B14" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
       <c r="C14" t="s">
-        <v>573</v>
+        <v>580</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>574</v>
+        <v>581</v>
       </c>
       <c r="B15" t="s">
-        <v>575</v>
+        <v>582</v>
       </c>
       <c r="C15" t="s">
-        <v>576</v>
+        <v>583</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="B16" t="s">
-        <v>578</v>
+        <v>585</v>
       </c>
       <c r="C16" t="s">
-        <v>579</v>
+        <v>586</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>580</v>
+        <v>587</v>
       </c>
       <c r="B17" t="s">
-        <v>581</v>
+        <v>588</v>
       </c>
       <c r="C17" t="s">
-        <v>582</v>
+        <v>589</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>584</v>
+        <v>591</v>
       </c>
       <c r="B20" t="s">
-        <v>585</v>
+        <v>592</v>
       </c>
       <c r="C20" t="s">
-        <v>586</v>
+        <v>593</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>587</v>
+        <v>594</v>
       </c>
       <c r="B21" t="s">
-        <v>588</v>
+        <v>595</v>
       </c>
       <c r="C21" t="s">
-        <v>589</v>
+        <v>596</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>590</v>
+        <v>597</v>
       </c>
       <c r="B22" t="s">
-        <v>591</v>
+        <v>598</v>
       </c>
       <c r="C22" t="s">
-        <v>592</v>
+        <v>599</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>593</v>
+        <v>600</v>
       </c>
       <c r="B23" t="s">
-        <v>594</v>
+        <v>601</v>
       </c>
       <c r="C23" t="s">
-        <v>595</v>
+        <v>602</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>596</v>
+        <v>603</v>
       </c>
       <c r="B24" t="s">
-        <v>597</v>
+        <v>604</v>
       </c>
       <c r="C24" t="s">
-        <v>598</v>
+        <v>605</v>
       </c>
     </row>
   </sheetData>

</xml_diff>